<commit_message>
Update dataset and site with expanded field list
</commit_message>
<xml_diff>
--- a/サバゲーフィールドDB_初期データ.xlsx
+++ b/サバゲーフィールドDB_初期データ.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:P58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3008,6 +3008,2086 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>千代田区(秋葉原)</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>ASOBIBA 秋葉原店</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>特になし(個人参加可)</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>秋葉原駅から徒歩4分、初心者大歓迎</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>https://asobiba-tokyo.com/fields/akihabara</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>江東区(新木場)</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>ASOBIBA 新木場</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>特になし(個人参加可)</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>新木場駅から徒歩7分、大型倉庫フィールド</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>https://asobiba-tokyo.com/fields/shinkiba</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>福生市</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>BLKFOX AIRSOFT FIELD 福生店</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>あり(無料)</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>福生駅西口から徒歩30秒、複雑に入り組んだCQBフィールド</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>https://blkfox.jp/</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>042-513-7003</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>八王子市</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>IBF9</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>2000年オープンの老舗インドアフィールド。屋外シューティングレンジ併設(50m×1/10m×4レーン)</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ibf9.com/</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>042-659-2898</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>千葉県</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>印西市</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>CIMAX</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>東京ドーム1個分の広さを誇る大型森林フィールド。バギー・キャンプ等も併設</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cimax.jp/</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>080-2730-0416</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>千葉県</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>印西市</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>ユニオンベース</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>建物が密集する市街地エリアと自然地形の高台を含む複合フィールド</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>https://union-base.com/</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>千葉県</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>千葉市中央区</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>STINGER</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>千葉駅から徒歩7分、6階建てビル全体を使う千葉県最大級インドアフィールド</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>http://www.stinger-survivalgame.com/</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>070-3665-7455</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>千葉県</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>千葉市花見川区</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>BATTLE</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>平日8:30〜17:30、休日・祝祭日8:00〜17:30営業</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.battle-airsoft.com/</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>埼玉県</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>入間市</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>ZEEK</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>フリーゲーム3,000円〜</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>2(A/Bフィールド)</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>さいたま最大級のインドアサバゲーフィールド。ショッピングプラザサイオス内</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>https://zeek-svg.com/</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>090-8108-9752</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>埼玉県</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>大里郡寄居町</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>CQBフォレスト</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>埼玉県寄居町の森林フィールド</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>https://cqbforest.com/</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>090-3599-7120</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>埼玉県</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>大里郡寄居町</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Rock254</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>市街地型で1万坪もの広大なフィールド</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>要確認(公式サイト不明、紹介サイト経由)</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>080-1985-0254</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>埼玉県</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>児玉郡美里町</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>アサルト3</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>埼玉最大級の森林フィールド</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>http://owl.main.jp/</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>090-6536-0799</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>神奈川県</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>逗子市</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>GARDEN-Z(ガーデンZ)</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>逗子・湘南エリアの山岳・平地を併せたフィールド。駐車場30台完備</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.garden-z.jp/</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>045-261-0013</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>神奈川県</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>相模原市緑区</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>九龍城 戦闘市街区</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>定例会9:00〜16:00 4,400円/1名</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>市街戦をイメージしたインドアフィールド</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>http://www.kowlooncity0801.com/index.html</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>神奈川県</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>横浜市都筑区</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>AREA41 横浜</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>港北みなも3F、都心アクセス良好</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>https://41px.jp/area41_yokohama/</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>茨城県</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>龍ケ崎市</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>サバイバルカントリー</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>200名(メインフィールド)</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>関東圏最大級の専有面積。定例会・イベントゲーム中心、200名収容のメインフィールド</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>https://survival-country.jp/</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>茨城県</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>小美玉市</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>フィールド小美鯖</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>3,000円または2,000円(初回+500円)</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>森林・CQBタイプ複合フィールド</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>https://omisaba.com/</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>090-4011-5444</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>茨城県</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>龍ケ崎市</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>つくばサバゲーランド</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>県下最大級。圏央道牛久阿見ICから10分、観戦台あり</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>https://coubic.com/tsukusaba</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>080-8066-8924</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>茨城県</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>牛久市</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>サバイバルゲームフィールド EDGE</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>総面積4,500坪の森林フィールド</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>https://sgf-edge.net/</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>茨城県</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>稲敷郡阿見町</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>サバゲーフィールドTEDO</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>全面アスファルトの金属バリケ主体CQBフィールド。3階建コンクリート廃墟あり</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tedo-svgf.com/</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>栃木県</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>那須郡那須町</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>サバゲパーク那須</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>要確認(貸切料金のみ判明)</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>予約制レンタルサバイバルゲーム＆レンタルフィールド</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>http://www.388nasu.com/</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>0287-63-3005</t>
+        </is>
+      </c>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>栃木県</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>芳賀郡市貝町</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Turf Battle Field</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>栃木県初、宿泊施設完備のサバゲーフィールド</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shinutsu.com/tbf/</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>群馬県</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>高崎市</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>ガンフィールド榛名</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>榛名山の麓にある広大な森林フィールド</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>https://unlimit-haruna.jp/gf-haruna/</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>070-6658-7630</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>群馬県</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>藤岡市</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>ASTREA(アストレア)</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>群馬県藤岡市のフィールド</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>要確認(公式サイト不明、サバゲーる経由)</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>0274-50-8688</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>群馬県</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>桐生市</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>AKAGI.357(赤城357)</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>赤城山麓のフィールド</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>https://akagi357.com/</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>080-4050-0357</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>関東</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>群馬県</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>桐生市</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>コンラードヒルズ</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>3,000円</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>栃木・群馬の県境エリアのフィールド。営業9時〜17時(17:30完全撤退)</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>https://c-hills.net/</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix Kanto field data quality and add BLKFOX Honatsugi
</commit_message>
<xml_diff>
--- a/サバゲーフィールドDB_初期データ.xlsx
+++ b/サバゲーフィールドDB_初期データ.xlsx
@@ -2454,22 +2454,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>関東</t>
+          <t>中部</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>埼玉県</t>
+          <t>長野県</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>比企郡滑川町</t>
+          <t>佐久市</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>サバっちゃアウトドア</t>
+          <t>アサルトフロント</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>3,000円</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2504,17 +2504,17 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>貸切専用、初心者・女性歓迎</t>
+          <t>長野県佐久市、木曜定休</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>https://sabaccha-outdoor.com/</t>
+          <t>要確認(公式サイト不明、紹介サイト経由)</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>080-8037-8279</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
@@ -2534,27 +2534,27 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>関東</t>
+          <t>北海道・東北</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>埼玉県</t>
+          <t>福島県</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>ふじみ野市</t>
+          <t>郡山市</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Brave Point 埼玉店</t>
+          <t>STRONGER(ストロンガー)</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>屋内</t>
+          <t>屋外</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2584,17 +2584,17 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>関東最大級サバゲースタジオ、池袋・大宮から約30分</t>
+          <t>東北最大級・最古参の一つ。3,500坪、毎週日曜と第3火曜に定例会</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>https://saitama.brave-point.jp/</t>
+          <t>https://stronger-fukusima.jimdofree.com/</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>049-269-3301</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
@@ -2614,42 +2614,42 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>関東</t>
+          <t>九州</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>神奈川県</t>
+          <t>熊本県</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>横浜市西区</t>
+          <t>菊池郡大津町</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>ASOBIBA横浜駅前店</t>
+          <t>サバイバルゲームフィールド トータス</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>屋内</t>
+          <t>屋外</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>平日午前3,000円/午後3,500円、土日祝4,000円</t>
+          <t>男性2,500円/女性1,500円</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>特になし</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>あり(レンタル無料キャンペーン実施の場合あり、要最新確認)</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2664,17 +2664,17 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>横浜駅東口改札より徒歩2分</t>
+          <t>熊本県大津町のフィールド</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>https://asobiba-tokyo.com/fields/yokohama</t>
+          <t>https://tortoiseozu.amebaownd.com/</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>070-9005-7851</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
@@ -2699,17 +2699,17 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>神奈川県</t>
+          <t>埼玉県</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>厚木市</t>
+          <t>比企郡滑川町</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>みんなの森</t>
+          <t>サバっちゃアウトドア</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -2744,12 +2744,12 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>14,000坪の山林フィールド。森林・草原・川を活かしたジャングル戦</t>
+          <t>貸切専用、初心者・女性歓迎</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>https://minmori.com/</t>
+          <t>https://sabaccha-outdoor.com/</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
@@ -2774,32 +2774,32 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>中部</t>
+          <t>関東</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>長野県</t>
+          <t>埼玉県</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>佐久市</t>
+          <t>ふじみ野市</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>アサルトフロント</t>
+          <t>Brave Point 埼玉店</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>屋外</t>
+          <t>屋内</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>3,000円</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2824,17 +2824,17 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>長野県佐久市、木曜定休</t>
+          <t>関東最大級サバゲースタジオ、池袋・大宮から約30分</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>要確認(公式サイト不明、紹介サイト経由)</t>
+          <t>https://saitama.brave-point.jp/</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>080-8037-8279</t>
+          <t>049-269-3301</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
@@ -2854,42 +2854,42 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>北海道・東北</t>
+          <t>関東</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>福島県</t>
+          <t>神奈川県</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>郡山市</t>
+          <t>横浜市西区</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>STRONGER(ストロンガー)</t>
+          <t>ASOBIBA横浜駅前店</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>屋外</t>
+          <t>屋内</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>平日午前3,000円/午後3,500円、土日祝4,000円</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>特になし</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>あり(レンタル無料キャンペーン実施の場合あり、要最新確認)</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2904,12 +2904,12 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>東北最大級・最古参の一つ。3,500坪、毎週日曜と第3火曜に定例会</t>
+          <t>横浜駅東口改札より徒歩2分</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>https://stronger-fukusima.jimdofree.com/</t>
+          <t>https://asobiba-tokyo.com/fields/yokohama</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
@@ -2934,22 +2934,22 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>九州</t>
+          <t>関東</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>熊本県</t>
+          <t>神奈川県</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>菊池郡大津町</t>
+          <t>厚木市</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>サバイバルゲームフィールド トータス</t>
+          <t>みんなの森</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>男性2,500円/女性1,500円</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2984,17 +2984,17 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>熊本県大津町のフィールド</t>
+          <t>14,000坪の山林フィールド。森林・草原・川を活かしたジャングル戦</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>https://tortoiseozu.amebaownd.com/</t>
+          <t>https://minmori.com/</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>070-9005-7851</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
@@ -3024,12 +3024,12 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>千代田区(秋葉原)</t>
+          <t>江東区(新木場)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>ASOBIBA 秋葉原店</t>
+          <t>ASOBIBA 新木場</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -3039,12 +3039,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>要確認(貸切中心、料金は公式サイト参照)</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>特になし(個人参加可)</t>
+          <t>特になし(個人参加可、フリー参加戦開催時のみ)</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>1(倉庫型CQBフィールド)</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -3064,22 +3064,22 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>秋葉原駅から徒歩4分、初心者大歓迎</t>
+          <t>新木場駅から徒歩7分、海沿いの倉庫街にある王道CQBフィールド。原則貸切営業</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>https://asobiba-tokyo.com/fields/akihabara</t>
+          <t>https://asobiba-tokyo.com/fields/shinkiba</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>要確認(お問い合わせフォームのみ、電話対応なし)</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -3104,12 +3104,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>江東区(新木場)</t>
+          <t>福生市</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>ASOBIBA 新木場</t>
+          <t>BLKFOX AIRSOFT FIELD 福生店</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -3119,47 +3119,47 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>要確認(公式サイト参照)</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>特になし(個人参加可)</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>あり</t>
+          <t>あり(無料)</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>1(330坪)</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>最大70名</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>新木場駅から徒歩7分、大型倉庫フィールド</t>
+          <t>福生駅西口から徒歩1分、330坪・最大70名収容。2018年開業、地下フィールドで雨天/夏場も快適</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>https://asobiba-tokyo.com/fields/shinkiba</t>
+          <t>https://blkfox.jp/fussa/</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>042-513-7003</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
@@ -3179,17 +3179,17 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>東京都</t>
+          <t>神奈川県</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>福生市</t>
+          <t>厚木市</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>BLKFOX AIRSOFT FIELD 福生店</t>
+          <t>BLKFOX AIRSOFT FIELD 本厚木店</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>要確認(公式サイト参照)</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -3214,32 +3214,32 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>1(約34m×24m)</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>最大66名</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>福生駅西口から徒歩30秒、複雑に入り組んだCQBフィールド</t>
+          <t>本厚木駅から徒歩2分、約34m×24m・最大66名収容。2026年開業のBLKFOX第2号店</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>https://blkfox.jp/</t>
+          <t>https://blkfox.jp/honatsugi/</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>042-513-7003</t>
+          <t>046-204-8646</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06)</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>要確認(現金のみ、公式サイト参照)</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>2000年オープンの老舗インドアフィールド。屋外シューティングレンジ併設(50m×1/10m×4レーン)</t>
+          <t>2000年オープンの老舗インドアフィールド。屋外シューティングレンジ併設(50m×1レーン/10m×4レーン)</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -3439,12 +3439,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>要確認(料金改定中、公式サイト参照)</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>予約不要の飛び込み参加可な定例会あり</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>建物が密集する市街地エリアと自然地形の高台を含む複合フィールド</t>
+          <t>建物が密集する市街地エリアと自然地形の高台を含む複合フィールド。ジュニアガン戦・夜戦貸切・BBQプランあり</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
@@ -3474,12 +3474,12 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>0476-76-9617</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
@@ -3599,7 +3599,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>要確認(公式サイト「平日定例会注意事項/料金一覧」参照)</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>平日8:30〜17:30、休日・祝祭日8:00〜17:30営業</t>
+          <t>都心一近い大型サバゲフィールド。平坦な地形で初心者に最適、八千代台駅から無料送迎あり</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
@@ -3634,12 +3634,12 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>070-1448-0308</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>フリーゲーム3,000円〜</t>
+          <t>おためし定例会2,500円(初利用者・女性・学生、毎月第2土曜)</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>さいたま最大級のインドアサバゲーフィールド。ショッピングプラザサイオス内</t>
+          <t>さいたま最大級のインドアサバゲーフィールド。ショッピングプラザサイオス内、多彩な定期コンテンツあり</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>平日3,000円/休日3,500円(1日、半日は2,000〜2,500円)</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -3774,17 +3774,17 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>1(月1回レイアウト変更)</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>貸切定員60名まで(休日)</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>埼玉県寄居町の森林フィールド</t>
+          <t>月1回レイアウト変更、最低8分のインターバル保証、オートセーフティエリアあり</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
@@ -3799,7 +3799,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>休日:男性3,200円/女性・子供2,200円、平日:男性2,700円/女性・子供1,700円</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -3859,17 +3859,17 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>貸切最大33名(休日)</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>市街地型で1万坪もの広大なフィールド</t>
+          <t>市街地型で1万坪(約33,000㎡)、デザート・市街戦エリアを含む広大なフィールド</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>要確認(公式サイト不明、紹介サイト経由)</t>
+          <t>https://rock254.com/</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -3979,22 +3979,22 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>神奈川県</t>
+          <t>埼玉県</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>逗子市</t>
+          <t>本庄市(旧群馬県藤岡市より移転)</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>GARDEN-Z(ガーデンZ)</t>
+          <t>ASTREA(アストレア)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>屋外</t>
+          <t>屋内</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -4024,22 +4024,22 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>逗子・湘南エリアの山岳・平地を併せたフィールド。駐車場30台完備</t>
+          <t>2025年に群馬県藤岡市から埼玉県本庄市へ移転(旧貸主による物件売却が理由)。2Fシューティングレンジ併設</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>https://www.garden-z.jp/</t>
+          <t>要確認(公式サイト不明、SNS中心)</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>045-261-0013</t>
+          <t>0274-50-8688(移転前の番号、要確認)</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>WebSearch(2026-07-06、移転情報あり)</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -4064,22 +4064,22 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>相模原市緑区</t>
+          <t>逗子市</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>九龍城 戦闘市街区</t>
+          <t>GARDEN-Z(ガーデンZ)</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>屋内</t>
+          <t>屋外</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>定例会9:00〜16:00 4,400円/1名</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -4104,17 +4104,17 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>市街戦をイメージしたインドアフィールド</t>
+          <t>逗子・湘南エリアの山岳・平地を併せたフィールド。駐車場30台完備</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>http://www.kowlooncity0801.com/index.html</t>
+          <t>https://www.garden-z.jp/</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>045-261-0013</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
@@ -4144,12 +4144,12 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>横浜市都筑区</t>
+          <t>相模原市緑区</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>AREA41 横浜</t>
+          <t>九龍 戦闘市街区</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -4159,7 +4159,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>定例会9:00〜16:00 4,400円/1名</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -4184,17 +4184,17 @@
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>港北みなも3F、都心アクセス良好</t>
+          <t>香港の九龍城塞をイメージした三階層の立体構造インドアフィールド。月曜定休</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>https://41px.jp/area41_yokohama/</t>
+          <t>http://www.kowlooncity0801.com/index.html</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>042-703-6050</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr">
@@ -4219,27 +4219,27 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>茨城県</t>
+          <t>神奈川県</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>龍ケ崎市</t>
+          <t>横浜市都筑区</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>サバイバルカントリー</t>
+          <t>AREA41 横浜</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>屋外</t>
+          <t>屋内</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>平日フリー4,400円、ホリデーゲーム1部5,400円/2部4,400円</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -4259,17 +4259,17 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>200名(メインフィールド)</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>関東圏最大級の専有面積。定例会・イベントゲーム中心、200名収容のメインフィールド</t>
+          <t>港北みなも3F、都心アクセス良好。平日定期券あり</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>https://survival-country.jp/</t>
+          <t>https://41px.jp/area41_yokohama/</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -4304,12 +4304,12 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>小美玉市</t>
+          <t>龍ケ崎市</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>フィールド小美鯖</t>
+          <t>サバイバルカントリー</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>3,000円または2,000円(初回+500円)</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -4339,22 +4339,22 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>200名(メインフィールド)</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>森林・CQBタイプ複合フィールド</t>
+          <t>関東圏最大級の専有面積。定例会・イベントゲーム中心、200名収容のメインフィールド</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>https://omisaba.com/</t>
+          <t>https://survival-country.jp/</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>090-4011-5444</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="O49" s="2" t="inlineStr">
@@ -4384,12 +4384,12 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>龍ケ崎市</t>
+          <t>小美玉市</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>つくばサバゲーランド</t>
+          <t>フィールド小美鯖</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>3,000円または2,000円(初回+500円)</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -4424,22 +4424,22 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>県下最大級。圏央道牛久阿見ICから10分、観戦台あり</t>
+          <t>約2,700坪。フォレストゾーン・グラウンドゾーンなど複数エリアで自由にレイアウト変更可能</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>https://coubic.com/tsukusaba</t>
+          <t>https://omisaba.com/</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>080-8066-8924</t>
+          <t>090-4011-5444</t>
         </is>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
@@ -4464,12 +4464,12 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>牛久市</t>
+          <t>龍ケ崎市</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>サバイバルゲームフィールド EDGE</t>
+          <t>つくばサバゲーランド</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -4504,17 +4504,17 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>総面積4,500坪の森林フィールド</t>
+          <t>県下最大級。圏央道牛久阿見ICから10分、観戦台あり</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>https://sgf-edge.net/</t>
+          <t>https://coubic.com/tsukusaba</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>080-8066-8924</t>
         </is>
       </c>
       <c r="O51" s="2" t="inlineStr">
@@ -4544,12 +4544,12 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>稲敷郡阿見町</t>
+          <t>牛久市</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>サバゲーフィールドTEDO</t>
+          <t>サバイバルゲームフィールド EDGE</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -4559,7 +4559,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>平日男性2,500円/女性1,500円、休日男性3,300円/女性2,000円</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -4574,7 +4574,7 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>要確認(2ndフィールドあり)</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -4584,22 +4584,22 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>全面アスファルトの金属バリケ主体CQBフィールド。3階建コンクリート廃墟あり</t>
+          <t>総面積4,500坪の森林フィールド。運営会社:株式会社EDGE。牛久阿見ICから約3分</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>https://www.tedo-svgf.com/</t>
+          <t>https://sgf-edge.net/</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>050-3647-2373</t>
         </is>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -4619,17 +4619,17 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>栃木県</t>
+          <t>茨城県</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>那須郡那須町</t>
+          <t>稲敷郡阿見町</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>サバゲパーク那須</t>
+          <t>サバゲーフィールドTEDO</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>要確認(貸切料金のみ判明)</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -4664,22 +4664,22 @@
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>予約制レンタルサバイバルゲーム＆レンタルフィールド</t>
+          <t>全面アスファルトの金属バリケ主体CQBフィールド。3階建コンクリート廃墟あり、撮影利用も可能</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>http://www.388nasu.com/</t>
+          <t>https://www.tedo-svgf.com/</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>0287-63-3005</t>
+          <t>要確認(メールのみ tedosvgf@gmail.com)</t>
         </is>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -4704,12 +4704,12 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>芳賀郡市貝町</t>
+          <t>那須郡那須町</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Turf Battle Field</t>
+          <t>サバゲパーク那須</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -4719,7 +4719,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>要確認(貸切料金のみ判明)</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -4744,22 +4744,22 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>栃木県初、宿泊施設完備のサバゲーフィールド</t>
+          <t>予約制レンタルサバイバルゲーム＆レンタルフィールド。那須ICから車で5分</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>https://www.shinutsu.com/tbf/</t>
+          <t>http://www.388nasu.com/</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>0287-63-3005</t>
         </is>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
@@ -4779,17 +4779,17 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>群馬県</t>
+          <t>栃木県</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>高崎市</t>
+          <t>芳賀郡市貝町</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>ガンフィールド榛名</t>
+          <t>Turf Battle Field</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -4824,22 +4824,22 @@
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>榛名山の麓にある広大な森林フィールド</t>
+          <t>栃木県初、宿泊施設完備のサバゲーフィールド。新宇都宮カントリークラブ敷地内、送迎バスあり</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>https://unlimit-haruna.jp/gf-haruna/</t>
+          <t>https://www.shinutsu.com/tbf/</t>
         </is>
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>070-6658-7630</t>
+          <t>要確認(問い合わせフォームのみ)</t>
         </is>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
@@ -4864,17 +4864,17 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>藤岡市</t>
+          <t>高崎市</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>ASTREA(アストレア)</t>
+          <t>ガンフィールド榛名</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>屋内</t>
+          <t>屋外</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -4904,17 +4904,17 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>群馬県藤岡市のフィールド</t>
+          <t>榛名山の麓にある広大な森林フィールド</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>要確認(公式サイト不明、サバゲーる経由)</t>
+          <t>https://unlimit-haruna.jp/gf-haruna/</t>
         </is>
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>0274-50-8688</t>
+          <t>070-6658-7630</t>
         </is>
       </c>
       <c r="O56" s="2" t="inlineStr">
@@ -5044,12 +5044,12 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>要確認(定員30人前後)</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>電動ガン・バッテリー・マスク&amp;ゴーグル</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>栃木・群馬の県境エリアのフィールド。営業9時〜17時(17:30完全撤退)</t>
+          <t>栃木・群馬の県境エリア、廃墟跡を利用したフィールド。営業9時〜17時(17:30完全撤退)、定員30人前後</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
@@ -5074,12 +5074,12 @@
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>080-8720-1910</t>
         </is>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06 再確認)</t>
         </is>
       </c>
       <c r="P58" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Expand nationwide fields to 98 records
</commit_message>
<xml_diff>
--- a/サバゲーフィールドDB_初期データ.xlsx
+++ b/サバゲーフィールドDB_初期データ.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P58"/>
+  <dimension ref="A1:P99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>沖縄県うるま市、月曜定休、営業時間10:00〜18:00</t>
+          <t>沖縄県うるま市天願、月曜定休、営業時間10:00〜18:00</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -5083,6 +5083,3286 @@
         </is>
       </c>
       <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>関西</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>兵庫県</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>加古川市</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>加古川CQBサバゲフィールド</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>要確認(貸切料金のみ判明)</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>兵庫県加古川市の市街戦型CQBフィールド</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>https://cqb-hyogo.com/</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>関西</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>兵庫県</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>神崎郡福崎町</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>C.Q.B GHOST 福崎店</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>1名3,500円(税込、2名以上で開催)</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>2名以上</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>約600坪の廃工場を利用した屋内型CQBフィールド。18歳未満・高校生は定例会参加不可(親子サバゲーイベントのみ)</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cqb-ghost.com/fukusaki</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>公式サイト(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>関西</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>兵庫県</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>神戸市西区</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>C.Q.B GHOST 神戸店</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>1名3,500円(税込、6名以上で開催)</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>6名以上</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>貸切最大40名(土日祝)</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>第二神明玉津IC北へ約6分、敷地面積約2,200坪の市街型屋外CQBフィールド。18歳未満・高校生は定例会参加不可</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cqb-ghost.com/kobe</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>公式サイト(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>関西</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>奈良県</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>LAGGOON CITY(ラグーンシティ)</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>男性3,500円/女性2,500円/高校生〜大学生2,500円/10〜15歳1,500円</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>営業時間AM10:00〜PM23:00、定休日金曜日</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>https://laggooncity.sabsta.jp/</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>関西</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>奈良県</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>奈良市中ノ川町713</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>テクニカルフィールド BATTLEZONE</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>近鉄奈良駅・JR奈良駅より奈良交通バス「下中ノ川」停留所下車徒歩1分</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>http://battlezone.jp/</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>関西</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>滋賀県</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>撃ちすぎサバゲフィールド</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>事前予約3,000円/飛び入り4,000円</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>プレオープンした開拓中の屋外フィールド、面積約6,000坪。開門時間08:00〜17:00</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>https://uchisugi.com/</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>公式サイト(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>関西</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>滋賀県</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>草津市</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Bb 南草津店</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>ゴーグル・靴・軍手など無料貸出</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>7歳から楽しめる銀玉鉄砲・10歳以上用レンタルガンあり。24時間営業、年中無休</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>077-566-7719</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>関西</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>和歌山県</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>西牟婁郡白浜町</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>IKORA PARKS(イコラパークス)</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>3(YARORA/CQB JUNGLE BASE/PARK)</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>総敷地面積約2万坪、サバイバルゲーム場・BBQ場・シューティング場の複合アウトドアレジャー施設。南紀白浜</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>http://ikoraparks.jp/</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>080-3771-6647</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>公式サイト(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>関西</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>和歌山県</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>橋本市</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>バトルランド-1</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>初回利用時に会員証(500円)の発行が必要</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>http://bl.ord.cc/</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>080-3859-8106</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>中部</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>岐阜県</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>羽島郡岐南町</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>BIG GATE</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>DAY/NIGHT各3,500円、通し6,000円</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>要事前予約、公式サイトのRESERVA予約システムで予約可能</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>https://big-gate.jp/</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>中部</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>岐阜県</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>多治見市</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>ふぁくとりー</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>要確認(貸切料金のみ判明)</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>岐阜県多治見市の市街戦型CQBフィールド</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>https://tokyosavage.jp/fielddetails/detail/138</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>中部</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>新潟県</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>阿賀野市(サントピアワールド敷地内)</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>新潟サバイバルゲームフィールドSTG</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>サントピアワールド敷地内にあるサバイバルゲーム専用フィールド</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>https://niigata-stg.com/</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>中部</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>新潟県</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>要確認(燕三条エリア)</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>サバイバルゲームスクエア ストライフ 燕三条</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>オールレンタル可能</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>2(メイン/10禁)</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>大型インドアフィールド、メイン&amp;10禁フィールド、エアコンセーフティ完備</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P71" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>中部</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>山梨県</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>大月市笹子町</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>AGITO(アジト)</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>要確認(貸切料金のみ判明)</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>2(A/Bフィールド)</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>受付時間09:00〜21:00</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>https://svgr.jp/place/61</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>080-3459-2727</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>中部</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>山梨県</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>甲州市塩山</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>サバイバルゲームフィールド369</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>都心から90分でアクセス可能、初心者講習・更衣室完備</t>
+        </is>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sgfield369.com/</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P73" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>中部</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>山梨県</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>北杜市(清里)</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>CTC</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>屋内/屋外</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>レンタル銃・ゴーグル・グローブ完備(手ぶらOK)</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>山梨県内最大規模、旧商業施設を利用した複合フィールド、初心者講習会あり</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>https://ctc-field.jp/</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P74" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>中部</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>石川県</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>金沢市</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Black boar</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>丘陵地形を活かしたフィールド、積雪時でもプレイ可能</t>
+        </is>
+      </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P75" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>中部</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>富山県</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>砺波市</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>SKYBASE TOYAMA</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>富山県最大級のサバゲーフィールド、初心者・女性歓迎</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>https://skybasetoyama88.wixsite.com/website-1</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P76" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>中部</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>福井県</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>南条郡南越前町</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>AREA365</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>福井県唯一のサバゲーフィールド、フラットで見通しの良い広大な敷地</t>
+        </is>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P77" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>九州</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>佐賀県</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>三養基郡みやき町</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>山水グリーンフィールド</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>要確認(貸切料金のみ判明)</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>佐賀県みやき町のフィールド</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>https://tokyosavage.jp/fielddetails/detail/216</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P78" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>九州</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>佐賀県</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>佐賀市大和町</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>RAPIDS(ラピッツ)</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>要確認(貸切料金のみ判明)</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>インドアCQBフィールド</t>
+        </is>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>https://tokyosavage.jp/fielddetails/detail/400</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P79" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>九州</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>長崎県</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>佐世保市小佐々町</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>サバイバルゲームフィールド 遊人(ゆうじん)</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>1,500円(昼)/1,500円(夜戦)</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>事務所は佐世保市小佐々町田原、フィールドは平原地区</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>https://navinagasaki.com/0956-68-2110/</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>0956-68-2110</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P80" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>九州</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>長崎県</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>佐世保市</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>佐世保サバゲーフィールド フクロウ</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>2021年10月オープン</t>
+        </is>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sasebo-fuku-low.com/price</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P81" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>九州</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>大分県</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>杵築市山香町</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>CAMP御戦</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>大分県杵築市のフィールド</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>https://camp-onsen.com/</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>070-2619-5140</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P82" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>九州</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>大分県</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>速見郡日出町</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>SAAT</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>サバイバルゲームフィールド&amp;ガンショップ併設。営業時間:平日12:00〜19:00(ゲーム開催日10:00〜)、土日祝9:30〜19:00</t>
+        </is>
+      </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>https://www.saat-oita.com/</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P83" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>九州</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>宮崎県</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>西都市</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>エイトドラゴン</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>宮崎県西都市のフィールド</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>070-4769-1741</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P84" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>九州</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>鹿児島県</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>鹿児島市平川町</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>サバイバルゲームフィールド DRAGOON</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>鹿児島市のフィールド</t>
+        </is>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P85" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>北海道・東北</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>青森県</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>要確認(津軽地方)</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>NEKO-TEN!(ネコ-テン!)</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>自然の草木を利用した森林戦フィールド</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P86" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>北海道・東北</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>青森県</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>八戸市</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>サバイバルゲームフィールド area52</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>青森県八戸市のフィールド</t>
+        </is>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>https://area52hachinohe.website/</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P87" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>北海道・東北</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>岩手県</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>胆沢郡金ケ崎町</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Battle Field BALLISTA(バリスタ)</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>40名</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>2019年6月開業、平坦なバリケードタイプ、月2〜3回定例会開催、収容40名。岩手県で現在営業中の数少ないフィールドの一つ</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>https://www4.hp-ez.com/hp/ballista/</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>北海道・東北</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>山形県</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>要確認(蔵王)</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>SABAGE PARK ZAO No.990</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>山形県蔵王のアウトドアサバゲーフィールド</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P89" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>島根県</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>仁多郡奥出雲町</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>仁多フィールド</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>2,500円</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>島根県奥出雲町のフィールド</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>https://nitafield.militaryblog.jp/</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P90" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>島根県</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>松江市宍道町</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>宍道サバゲーPARK DANDAN</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>島根県松江市宍道町のフィールド</t>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P91" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>鳥取県</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>西伯郡大山町</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>AIRSOFT DEYS</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>鳥取県大山町のフィールド</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P92" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>山口県</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>宇部市藤河内</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>宇部アウトドアフィールド &amp;GREEN</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>山口県宇部市のフィールド</t>
+        </is>
+      </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P93" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>四国</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>徳島県</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>徳島市国府町</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>C.Q.B FIELD ALPHA(アルファ)</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>土日祝3,000円(女性2,000円)/平日2,000円(女性1,500円)</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>営業時間10:00〜22:00</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>https://tokyosavage.jp/fielddetails/detail/331</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>080-4030-4127</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P94" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>四国</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>高知県</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>高知市春野町</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>ジャブロ(JABRO)</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>複合的サバイバルゲームフィールド</t>
+        </is>
+      </c>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>https://jabro.xyz/</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>080-4998-0079</t>
+        </is>
+      </c>
+      <c r="O95" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P95" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>四国</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>高知県</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>E.W.C(エキサイティングスポーツフィールド ホワイトクロー)</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>2024年6月に屋内サバイバルゲームフィールドとして誕生</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P96" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>沖縄</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>沖縄県</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>中頭郡中城村</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>オキナワエアソフトパーク(OAG)</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>営業時間10:00〜18:00(土曜のみ10:00〜23:00)、定休日不定休</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oag2010.com/field.php</t>
+        </is>
+      </c>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>080-9141-5515</t>
+        </is>
+      </c>
+      <c r="O97" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P97" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>沖縄</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>沖縄県</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>豊見城市</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>J.COMPACT</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>屋外</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>2024年12月1日オープン</t>
+        </is>
+      </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P98" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>沖縄</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>沖縄県</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>中頭郡読谷村</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>RBO field</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>屋内</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>2025年2月26日オープンしたインドアフィールド</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="O99" s="2" t="inlineStr">
+        <is>
+          <t>WebSearch(2026-07-06)</t>
+        </is>
+      </c>
+      <c r="P99" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>

</xml_diff>

<commit_message>
Fill in remaining 要確認 data for regional records, remove closed CTC field (97 records)
</commit_message>
<xml_diff>
--- a/サバゲーフィールドDB_初期データ.xlsx
+++ b/サバゲーフィールドDB_初期データ.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P99"/>
+  <dimension ref="A1:P98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5344,7 +5344,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>天理市稲葉町66-1</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>定員60名(夜戦は40名)</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -5374,17 +5374,17 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>1(全面アスファルト市街地型)</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>定例会定員60名/夜戦40名</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>営業時間AM10:00〜PM23:00、定休日金曜日</t>
+          <t>全面アスファルトの市街地型CQBフィールド(2,000㎡以上)。営業時間AM9:00〜PM17:00。土日祝・平日定例会(定員60名)、夜戦(定員40名)、KIDS WARあり</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
@@ -5399,7 +5399,7 @@
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06)</t>
         </is>
       </c>
       <c r="P62" s="2" t="inlineStr">
@@ -5824,7 +5824,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>羽島郡岐南町</t>
+          <t>羽島郡岐南町野中6丁目92-1</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -5849,22 +5849,22 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>10・18禁レンタル銃あり(有料)、ゴーグル・フェイスマスク無料</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>1(CQBエリア+競技エリア)</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>駐車場18台(最大30台)、席数28席</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>要事前予約、公式サイトのRESERVA予約システムで予約可能</t>
+          <t>インドア工場型CQBフィールド(推奨6vs6)+ASPカップ/スティールチャレンジ競技エリア併設。要事前予約</t>
         </is>
       </c>
       <c r="M68" s="2" t="inlineStr">
@@ -5874,12 +5874,12 @@
       </c>
       <c r="N68" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>090-3834-5177</t>
         </is>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06)</t>
         </is>
       </c>
       <c r="P68" s="2" t="inlineStr">
@@ -5984,7 +5984,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>阿賀野市(サントピアワールド敷地内)</t>
+          <t>阿賀野市保田486(遊園地サントピアワールド敷地内)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -6009,7 +6009,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>レンタル銃多数あり</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -6024,7 +6024,7 @@
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>サントピアワールド敷地内にあるサバイバルゲーム専用フィールド</t>
+          <t>2022年春開業。遊園地サントピアワールド敷地内。女性割引あり、貸切対応可</t>
         </is>
       </c>
       <c r="M70" s="2" t="inlineStr">
@@ -6039,7 +6039,7 @@
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06)</t>
         </is>
       </c>
       <c r="P70" s="2" t="inlineStr">
@@ -6299,22 +6299,22 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>山梨県</t>
+          <t>石川県</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>北杜市(清里)</t>
+          <t>金沢市</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>CTC</t>
+          <t>Black boar</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>屋内/屋外</t>
+          <t>屋外</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -6329,7 +6329,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>レンタル銃・ゴーグル・グローブ完備(手ぶらOK)</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -6344,12 +6344,12 @@
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>山梨県内最大規模、旧商業施設を利用した複合フィールド、初心者講習会あり</t>
+          <t>丘陵地形を活かしたフィールド、積雪時でもプレイ可能</t>
         </is>
       </c>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>https://ctc-field.jp/</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="N74" s="2" t="inlineStr">
@@ -6379,17 +6379,17 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>石川県</t>
+          <t>富山県</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>金沢市</t>
+          <t>砺波市</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Black boar</t>
+          <t>SKYBASE TOYAMA</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -6424,12 +6424,12 @@
       </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>丘陵地形を活かしたフィールド、積雪時でもプレイ可能</t>
+          <t>富山県最大級のサバゲーフィールド、初心者・女性歓迎</t>
         </is>
       </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>https://skybasetoyama88.wixsite.com/website-1</t>
         </is>
       </c>
       <c r="N75" s="2" t="inlineStr">
@@ -6459,17 +6459,17 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>富山県</t>
+          <t>福井県</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>砺波市</t>
+          <t>南条郡南越前町</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>SKYBASE TOYAMA</t>
+          <t>AREA365</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -6504,12 +6504,12 @@
       </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>富山県最大級のサバゲーフィールド、初心者・女性歓迎</t>
+          <t>福井県唯一のサバゲーフィールド、フラットで見通しの良い広大な敷地</t>
         </is>
       </c>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>https://skybasetoyama88.wixsite.com/website-1</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="N76" s="2" t="inlineStr">
@@ -6534,22 +6534,22 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>中部</t>
+          <t>九州</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>福井県</t>
+          <t>佐賀県</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>南条郡南越前町</t>
+          <t>三養基郡みやき町大字蓑原4807</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>AREA365</t>
+          <t>山水グリーンフィールド</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -6559,7 +6559,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>2,000円</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -6569,12 +6569,12 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>あり</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>2(第一/第二フィールド)</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr">
@@ -6584,12 +6584,12 @@
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>福井県唯一のサバゲーフィールド、フラットで見通しの良い広大な敷地</t>
+          <t>全長130m×幅40mの第一フィールドと全長200m×幅100mの第二フィールドの2面運営。シャワー完備、18歳未満参加可</t>
         </is>
       </c>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>http://kokusimusou5963.wixsite.com/sansui</t>
         </is>
       </c>
       <c r="N77" s="2" t="inlineStr">
@@ -6599,7 +6599,7 @@
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>サバゲーナビ(2026-07-06)</t>
         </is>
       </c>
       <c r="P77" s="2" t="inlineStr">
@@ -6624,22 +6624,22 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>三養基郡みやき町</t>
+          <t>佐賀市大和町大字松瀬4248-25</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>山水グリーンフィールド</t>
+          <t>RAPIDS(ラピッツ)</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>屋外</t>
+          <t>屋内</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>要確認(貸切料金のみ判明)</t>
+          <t>2,500円</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -6649,27 +6649,27 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>あり</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>2(アウト/インドア)</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>アウト40名/インドア30名</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>佐賀県みやき町のフィールド</t>
+          <t>アウトドア・インドア併設の複合フィールド、雨天時も利用可。18歳未満参加不可、駐車場40台</t>
         </is>
       </c>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>https://tokyosavage.jp/fielddetails/detail/216</t>
+          <t>https://asarapids.jimdofree.com/</t>
         </is>
       </c>
       <c r="N78" s="2" t="inlineStr">
@@ -6679,7 +6679,7 @@
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>サバゲーナビ(2026-07-06)</t>
         </is>
       </c>
       <c r="P78" s="2" t="inlineStr">
@@ -6699,27 +6699,27 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>佐賀県</t>
+          <t>長崎県</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>佐賀市大和町</t>
+          <t>佐世保市小佐々町</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>RAPIDS(ラピッツ)</t>
+          <t>サバイバルゲームフィールド 遊人(ゆうじん)</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>屋内</t>
+          <t>屋外</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>要確認(貸切料金のみ判明)</t>
+          <t>1,500円(昼)/1,500円(夜戦)</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -6744,17 +6744,17 @@
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>インドアCQBフィールド</t>
+          <t>事務所は佐世保市小佐々町田原、フィールドは平原地区</t>
         </is>
       </c>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>https://tokyosavage.jp/fielddetails/detail/400</t>
+          <t>https://navinagasaki.com/0956-68-2110/</t>
         </is>
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>0956-68-2110</t>
         </is>
       </c>
       <c r="O79" s="2" t="inlineStr">
@@ -6784,12 +6784,12 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>佐世保市小佐々町</t>
+          <t>佐世保市指方町1351</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>サバイバルゲームフィールド 遊人(ゆうじん)</t>
+          <t>佐世保サバゲーフィールド フクロウ</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -6799,7 +6799,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>1,500円(昼)/1,500円(夜戦)</t>
+          <t>DAY/NIGHT各3,000円</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -6809,7 +6809,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>レンタル銃2,000円、ゴーグル・マスク等無料貸出多数</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -6824,22 +6824,22 @@
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>事務所は佐世保市小佐々町田原、フィールドは平原地区</t>
+          <t>定休日木曜日。18歳未満は保護者同伴のみ参加可。シューティングレンジ併設</t>
         </is>
       </c>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>https://navinagasaki.com/0956-68-2110/</t>
+          <t>https://www.sasebo-fuku-low.com/price</t>
         </is>
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>0956-68-2110</t>
+          <t>090-1253-2960</t>
         </is>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06)</t>
         </is>
       </c>
       <c r="P80" s="2" t="inlineStr">
@@ -6859,17 +6859,17 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>長崎県</t>
+          <t>大分県</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>佐世保市</t>
+          <t>杵築市山香町大字野原3-4657-182</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>佐世保サバゲーフィールド フクロウ</t>
+          <t>CAMP御戦</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -6904,22 +6904,22 @@
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>2021年10月オープン</t>
+          <t>CQBと森の複合型フィールド。休憩所は駐車場から近く、夏は扇風機・冬は薪ストーブあり。毎週日曜フリー参加デー開催</t>
         </is>
       </c>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>https://www.sasebo-fuku-low.com/price</t>
+          <t>https://camp-onsen.com/</t>
         </is>
       </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>070-2619-5140</t>
         </is>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06)</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr">
@@ -6944,12 +6944,12 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>杵築市山香町</t>
+          <t>速見郡日出町豊岡1830-2</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>CAMP御戦</t>
+          <t>SAAT</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -6969,7 +6969,7 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>あり</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -6984,22 +6984,22 @@
       </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>大分県杵築市のフィールド</t>
+          <t>ガンショップ併設、2,000坪のアウトドア型フィールド。45mシューティングレンジ完備。営業時間:平日12:00〜19:00(ゲーム開催日9:30〜)、土日祝9:30〜19:00</t>
         </is>
       </c>
       <c r="M82" s="2" t="inlineStr">
         <is>
-          <t>https://camp-onsen.com/</t>
+          <t>https://www.saat-oita.com/</t>
         </is>
       </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>070-2619-5140</t>
+          <t>0977-76-8977</t>
         </is>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06)</t>
         </is>
       </c>
       <c r="P82" s="2" t="inlineStr">
@@ -7019,17 +7019,17 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>大分県</t>
+          <t>宮崎県</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>速見郡日出町</t>
+          <t>西都市</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>SAAT</t>
+          <t>エイトドラゴン</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -7064,17 +7064,17 @@
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>サバイバルゲームフィールド&amp;ガンショップ併設。営業時間:平日12:00〜19:00(ゲーム開催日10:00〜)、土日祝9:30〜19:00</t>
+          <t>宮崎県西都市のフィールド</t>
         </is>
       </c>
       <c r="M83" s="2" t="inlineStr">
         <is>
-          <t>https://www.saat-oita.com/</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>070-4769-1741</t>
         </is>
       </c>
       <c r="O83" s="2" t="inlineStr">
@@ -7099,17 +7099,17 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>宮崎県</t>
+          <t>鹿児島県</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>西都市</t>
+          <t>鹿児島市平川町</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>エイトドラゴン</t>
+          <t>サバイバルゲームフィールド DRAGOON</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -7144,7 +7144,7 @@
       </c>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>宮崎県西都市のフィールド</t>
+          <t>鹿児島市のフィールド</t>
         </is>
       </c>
       <c r="M84" s="2" t="inlineStr">
@@ -7154,7 +7154,7 @@
       </c>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>070-4769-1741</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="O84" s="2" t="inlineStr">
@@ -7174,22 +7174,22 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>九州</t>
+          <t>北海道・東北</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>鹿児島県</t>
+          <t>青森県</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>鹿児島市平川町</t>
+          <t>要確認(津軽地方)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>サバイバルゲームフィールド DRAGOON</t>
+          <t>NEKO-TEN!(ネコ-テン!)</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>鹿児島市のフィールド</t>
+          <t>自然の草木を利用した森林戦フィールド</t>
         </is>
       </c>
       <c r="M85" s="2" t="inlineStr">
@@ -7264,12 +7264,12 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>要確認(津軽地方)</t>
+          <t>八戸市</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>NEKO-TEN!(ネコ-テン!)</t>
+          <t>サバイバルゲームフィールド area52</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -7284,12 +7284,12 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>10歳以上、予約不要</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>レンタルガンあり</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -7304,22 +7304,22 @@
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>自然の草木を利用した森林戦フィールド</t>
+          <t>毎週日曜「サバゲーやるデー」開催、10歳以上なら予約不要で参加OK。貸切・夜戦も対応</t>
         </is>
       </c>
       <c r="M86" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>https://area52hachinohe.website/</t>
         </is>
       </c>
       <c r="N86" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>080-6000-5214</t>
         </is>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>公式サイト(2026-07-06)</t>
         </is>
       </c>
       <c r="P86" s="2" t="inlineStr">
@@ -7339,17 +7339,17 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>青森県</t>
+          <t>岩手県</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>八戸市</t>
+          <t>胆沢郡金ケ崎町</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>サバイバルゲームフィールド area52</t>
+          <t>Battle Field BALLISTA(バリスタ)</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -7379,17 +7379,17 @@
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>40名</t>
         </is>
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>青森県八戸市のフィールド</t>
+          <t>2019年6月開業、平坦なバリケードタイプ、月2〜3回定例会開催、収容40名。岩手県で現在営業中の数少ないフィールドの一つ</t>
         </is>
       </c>
       <c r="M87" s="2" t="inlineStr">
         <is>
-          <t>https://area52hachinohe.website/</t>
+          <t>https://www4.hp-ez.com/hp/ballista/</t>
         </is>
       </c>
       <c r="N87" s="2" t="inlineStr">
@@ -7419,17 +7419,17 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>岩手県</t>
+          <t>山形県</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>胆沢郡金ケ崎町</t>
+          <t>要確認(蔵王)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Battle Field BALLISTA(バリスタ)</t>
+          <t>SABAGE PARK ZAO No.990</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -7459,17 +7459,17 @@
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>40名</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>2019年6月開業、平坦なバリケードタイプ、月2〜3回定例会開催、収容40名。岩手県で現在営業中の数少ないフィールドの一つ</t>
+          <t>山形県蔵王のアウトドアサバゲーフィールド</t>
         </is>
       </c>
       <c r="M88" s="2" t="inlineStr">
         <is>
-          <t>https://www4.hp-ez.com/hp/ballista/</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="N88" s="2" t="inlineStr">
@@ -7494,22 +7494,22 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>北海道・東北</t>
+          <t>中国</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>山形県</t>
+          <t>島根県</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>要確認(蔵王)</t>
+          <t>仁多郡奥出雲町</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>SABAGE PARK ZAO No.990</t>
+          <t>仁多フィールド</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>2,500円</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -7544,12 +7544,12 @@
       </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>山形県蔵王のアウトドアサバゲーフィールド</t>
+          <t>島根県奥出雲町のフィールド</t>
         </is>
       </c>
       <c r="M89" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>https://nitafield.militaryblog.jp/</t>
         </is>
       </c>
       <c r="N89" s="2" t="inlineStr">
@@ -7584,12 +7584,12 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>仁多郡奥出雲町</t>
+          <t>松江市宍道町</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>仁多フィールド</t>
+          <t>宍道サバゲーPARK DANDAN</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -7599,7 +7599,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>2,500円</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -7624,12 +7624,12 @@
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>島根県奥出雲町のフィールド</t>
+          <t>島根県松江市宍道町のフィールド</t>
         </is>
       </c>
       <c r="M90" s="2" t="inlineStr">
         <is>
-          <t>https://nitafield.militaryblog.jp/</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="N90" s="2" t="inlineStr">
@@ -7659,17 +7659,17 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>島根県</t>
+          <t>鳥取県</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>松江市宍道町</t>
+          <t>西伯郡大山町</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>宍道サバゲーPARK DANDAN</t>
+          <t>AIRSOFT DEYS</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -7704,7 +7704,7 @@
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>島根県松江市宍道町のフィールド</t>
+          <t>鳥取県大山町のフィールド</t>
         </is>
       </c>
       <c r="M91" s="2" t="inlineStr">
@@ -7739,17 +7739,17 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>鳥取県</t>
+          <t>山口県</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>西伯郡大山町</t>
+          <t>宇部市藤河内</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>AIRSOFT DEYS</t>
+          <t>宇部アウトドアフィールド &amp;GREEN</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -7784,7 +7784,7 @@
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>鳥取県大山町のフィールド</t>
+          <t>山口県宇部市のフィールド</t>
         </is>
       </c>
       <c r="M92" s="2" t="inlineStr">
@@ -7814,22 +7814,22 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>中国</t>
+          <t>四国</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>山口県</t>
+          <t>徳島県</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>宇部市藤河内</t>
+          <t>徳島市国府町早淵843</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>宇部アウトドアフィールド &amp;GREEN</t>
+          <t>C.Q.B FIELD ALPHA(アルファ)</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>土日祝3,000円(女性2,000円)/平日2,000円(女性1,500円)</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -7849,7 +7849,7 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>あり</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -7859,27 +7859,27 @@
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>貸切最大20名(土日祝)</t>
         </is>
       </c>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t>山口県宇部市のフィールド</t>
+          <t>バリケード構成のCQBフィールド。18歳未満参加不可、駐車場30台</t>
         </is>
       </c>
       <c r="M93" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>https://cqbfieldalpha.wixsite.com/timber</t>
         </is>
       </c>
       <c r="N93" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>080-4030-4127</t>
         </is>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>WebSearch(2026-07-06)</t>
+          <t>サバゲーナビ(2026-07-06)</t>
         </is>
       </c>
       <c r="P93" s="2" t="inlineStr">
@@ -7899,27 +7899,27 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>徳島県</t>
+          <t>高知県</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>徳島市国府町</t>
+          <t>高知市春野町</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>C.Q.B FIELD ALPHA(アルファ)</t>
+          <t>ジャブロ(JABRO)</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>屋内</t>
+          <t>屋外</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>土日祝3,000円(女性2,000円)/平日2,000円(女性1,500円)</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -7944,17 +7944,17 @@
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>営業時間10:00〜22:00</t>
+          <t>複合的サバイバルゲームフィールド</t>
         </is>
       </c>
       <c r="M94" s="2" t="inlineStr">
         <is>
-          <t>https://tokyosavage.jp/fielddetails/detail/331</t>
+          <t>https://jabro.xyz/</t>
         </is>
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>080-4030-4127</t>
+          <t>080-4998-0079</t>
         </is>
       </c>
       <c r="O94" s="2" t="inlineStr">
@@ -7984,17 +7984,17 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>高知市春野町</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>ジャブロ(JABRO)</t>
+          <t>E.W.C(エキサイティングスポーツフィールド ホワイトクロー)</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>屋外</t>
+          <t>屋内</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -8024,17 +8024,17 @@
       </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t>複合的サバイバルゲームフィールド</t>
+          <t>2024年6月に屋内サバイバルゲームフィールドとして誕生</t>
         </is>
       </c>
       <c r="M95" s="2" t="inlineStr">
         <is>
-          <t>https://jabro.xyz/</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="N95" s="2" t="inlineStr">
         <is>
-          <t>080-4998-0079</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="O95" s="2" t="inlineStr">
@@ -8054,27 +8054,27 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>四国</t>
+          <t>沖縄</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>高知県</t>
+          <t>沖縄県</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>中頭郡中城村</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>E.W.C(エキサイティングスポーツフィールド ホワイトクロー)</t>
+          <t>オキナワエアソフトパーク(OAG)</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>屋内</t>
+          <t>屋外</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -8104,17 +8104,17 @@
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>2024年6月に屋内サバイバルゲームフィールドとして誕生</t>
+          <t>営業時間10:00〜18:00(土曜のみ10:00〜23:00)、定休日不定休</t>
         </is>
       </c>
       <c r="M96" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>https://www.oag2010.com/field.php</t>
         </is>
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>080-9141-5515</t>
         </is>
       </c>
       <c r="O96" s="2" t="inlineStr">
@@ -8144,12 +8144,12 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>中頭郡中城村</t>
+          <t>豊見城市</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>オキナワエアソフトパーク(OAG)</t>
+          <t>J.COMPACT</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -8184,17 +8184,17 @@
       </c>
       <c r="L97" s="2" t="inlineStr">
         <is>
-          <t>営業時間10:00〜18:00(土曜のみ10:00〜23:00)、定休日不定休</t>
+          <t>2024年12月1日オープン</t>
         </is>
       </c>
       <c r="M97" s="2" t="inlineStr">
         <is>
-          <t>https://www.oag2010.com/field.php</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="N97" s="2" t="inlineStr">
         <is>
-          <t>080-9141-5515</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="O97" s="2" t="inlineStr">
@@ -8224,17 +8224,17 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>豊見城市</t>
+          <t>中頭郡読谷村</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>J.COMPACT</t>
+          <t>RBO field</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>屋外</t>
+          <t>屋内</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="L98" s="2" t="inlineStr">
         <is>
-          <t>2024年12月1日オープン</t>
+          <t>2025年2月26日オープンしたインドアフィールド</t>
         </is>
       </c>
       <c r="M98" s="2" t="inlineStr">
@@ -8283,86 +8283,6 @@
         </is>
       </c>
       <c r="P98" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="B99" s="2" t="inlineStr">
-        <is>
-          <t>沖縄</t>
-        </is>
-      </c>
-      <c r="C99" s="2" t="inlineStr">
-        <is>
-          <t>沖縄県</t>
-        </is>
-      </c>
-      <c r="D99" s="2" t="inlineStr">
-        <is>
-          <t>中頭郡読谷村</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
-          <t>RBO field</t>
-        </is>
-      </c>
-      <c r="F99" s="2" t="inlineStr">
-        <is>
-          <t>屋内</t>
-        </is>
-      </c>
-      <c r="G99" s="2" t="inlineStr">
-        <is>
-          <t>要確認</t>
-        </is>
-      </c>
-      <c r="H99" s="2" t="inlineStr">
-        <is>
-          <t>要確認</t>
-        </is>
-      </c>
-      <c r="I99" s="2" t="inlineStr">
-        <is>
-          <t>要確認</t>
-        </is>
-      </c>
-      <c r="J99" s="2" t="inlineStr">
-        <is>
-          <t>要確認</t>
-        </is>
-      </c>
-      <c r="K99" s="2" t="inlineStr">
-        <is>
-          <t>要確認</t>
-        </is>
-      </c>
-      <c r="L99" s="2" t="inlineStr">
-        <is>
-          <t>2025年2月26日オープンしたインドアフィールド</t>
-        </is>
-      </c>
-      <c r="M99" s="2" t="inlineStr">
-        <is>
-          <t>要確認</t>
-        </is>
-      </c>
-      <c r="N99" s="2" t="inlineStr">
-        <is>
-          <t>要確認</t>
-        </is>
-      </c>
-      <c r="O99" s="2" t="inlineStr">
-        <is>
-          <t>WebSearch(2026-07-06)</t>
-        </is>
-      </c>
-      <c r="P99" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>

</xml_diff>

<commit_message>
Fix meeting_fee display for JABRO and E.W.C
</commit_message>
<xml_diff>
--- a/サバゲーフィールドDB_初期データ.xlsx
+++ b/サバゲーフィールドDB_初期データ.xlsx
@@ -7903,7 +7903,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>貸切のみ:平日20,000円〜(6名まで)</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>平日2,000円〜/休日2,000円〜(時間帯制)</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">

</xml_diff>